<commit_message>
Update portal data and pages
</commit_message>
<xml_diff>
--- a/activitereeldirect-2026.xlsx
+++ b/activitereeldirect-2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\OneDrive\Bureau\CODE HTML\Developpements\APP KENT VERCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE24AF0F-0E11-4056-AC56-4D65E90EB418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38BB671-B2A7-4E4F-BB6F-FDCA87389928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{52F3EE67-8AA3-4B10-A5A9-DE88DE815FD5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="107">
   <si>
     <t>N°commande</t>
   </si>
@@ -345,6 +345,18 @@
   </si>
   <si>
     <t>Mars</t>
+  </si>
+  <si>
+    <t>26404913</t>
+  </si>
+  <si>
+    <t>26605307</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDE KEVIN                </t>
+  </si>
+  <si>
+    <t>Février</t>
   </si>
 </sst>
 </file>
@@ -720,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA07812-0C85-468D-8FD3-167ED09F5A69}">
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:W18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.35">
@@ -1788,6 +1800,219 @@
         <v>102</v>
       </c>
     </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16" s="1">
+        <v>46071</v>
+      </c>
+      <c r="G16" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" t="s">
+        <v>59</v>
+      </c>
+      <c r="I16" t="s">
+        <v>60</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <v>85.68</v>
+      </c>
+      <c r="L16">
+        <v>85.68</v>
+      </c>
+      <c r="M16" t="s">
+        <v>29</v>
+      </c>
+      <c r="N16" t="s">
+        <v>30</v>
+      </c>
+      <c r="O16" s="1">
+        <v>46071</v>
+      </c>
+      <c r="P16" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>32</v>
+      </c>
+      <c r="R16" t="s">
+        <v>33</v>
+      </c>
+      <c r="S16" t="s">
+        <v>34</v>
+      </c>
+      <c r="T16" t="s">
+        <v>61</v>
+      </c>
+      <c r="U16" t="s">
+        <v>62</v>
+      </c>
+      <c r="V16" t="s">
+        <v>63</v>
+      </c>
+      <c r="W16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="1">
+        <v>46071</v>
+      </c>
+      <c r="G17" t="s">
+        <v>67</v>
+      </c>
+      <c r="H17" t="s">
+        <v>68</v>
+      </c>
+      <c r="I17" t="s">
+        <v>69</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>247.96</v>
+      </c>
+      <c r="L17">
+        <v>247.96</v>
+      </c>
+      <c r="M17" t="s">
+        <v>29</v>
+      </c>
+      <c r="N17" t="s">
+        <v>30</v>
+      </c>
+      <c r="O17" s="1">
+        <v>46071</v>
+      </c>
+      <c r="P17" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>32</v>
+      </c>
+      <c r="R17" t="s">
+        <v>33</v>
+      </c>
+      <c r="S17" t="s">
+        <v>34</v>
+      </c>
+      <c r="T17" t="s">
+        <v>61</v>
+      </c>
+      <c r="U17" t="s">
+        <v>62</v>
+      </c>
+      <c r="V17" t="s">
+        <v>63</v>
+      </c>
+      <c r="W17" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" t="s">
+        <v>57</v>
+      </c>
+      <c r="F18" s="1">
+        <v>46071</v>
+      </c>
+      <c r="G18" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" t="s">
+        <v>87</v>
+      </c>
+      <c r="J18">
+        <v>3</v>
+      </c>
+      <c r="K18">
+        <v>25.44</v>
+      </c>
+      <c r="L18">
+        <v>76.319999999999993</v>
+      </c>
+      <c r="M18" t="s">
+        <v>29</v>
+      </c>
+      <c r="N18" t="s">
+        <v>30</v>
+      </c>
+      <c r="O18" s="1">
+        <v>46071</v>
+      </c>
+      <c r="P18" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>32</v>
+      </c>
+      <c r="R18" t="s">
+        <v>33</v>
+      </c>
+      <c r="S18" t="s">
+        <v>34</v>
+      </c>
+      <c r="T18" t="s">
+        <v>61</v>
+      </c>
+      <c r="U18" t="s">
+        <v>62</v>
+      </c>
+      <c r="V18" t="s">
+        <v>63</v>
+      </c>
+      <c r="W18" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>